<commit_message>
Replace sample import workbook with realistic cross-linked operations demo data
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/dashboard/assets/SBS_operations_sample.xlsx
+++ b/dashboard/assets/SBS_operations_sample.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -448,31 +448,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TR-SAMPLE01</v>
+        <v>TR-2026-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Sample Trainee</v>
+        <v>Nour El-Din Hassan</v>
       </c>
       <c r="C2" t="str">
-        <v>+1000000000</v>
+        <v>+20 100 222 3344</v>
       </c>
       <c r="D2" t="str">
-        <v>sample.trainee@example.com</v>
+        <v>nour.hassan@example.org</v>
       </c>
       <c r="E2" t="str">
-        <v>Doctor</v>
+        <v>Physician</v>
       </c>
       <c r="F2" t="str">
-        <v>Sample Co</v>
+        <v>Cairo University Hospital</v>
       </c>
       <c r="G2" t="str">
-        <v>Analyst</v>
+        <v>Resident</v>
       </c>
       <c r="H2" t="str">
-        <v>Sample University</v>
+        <v>Cairo University</v>
       </c>
       <c r="I2" t="str">
-        <v>General</v>
+        <v>Internal Medicine</v>
       </c>
       <c r="J2" t="str">
         <v>Cairo</v>
@@ -481,42 +481,42 @@
         <v/>
       </c>
       <c r="L2" t="str">
-        <v>2026-01-15</v>
+        <v>2026-01-08</v>
       </c>
       <c r="M2" t="str">
         <v>Active</v>
       </c>
       <c r="N2" t="str">
-        <v>Demo import row</v>
+        <v>Demo: enrolled in leadership batch</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>TR-SAMPLE02</v>
+        <v>TR-2026-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Second Trainee</v>
+        <v>Sara Mahmoud Fathy</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>+20 101 333 4455</v>
       </c>
       <c r="D3" t="str">
-        <v>second@example.com</v>
+        <v>sara.mahmoud@example.org</v>
       </c>
       <c r="E3" t="str">
-        <v>Student</v>
+        <v>Pharmacist</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>Alexandria Health Directorate</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>Clinical Pharmacist</v>
       </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>Hospital Pharmacy</v>
       </c>
       <c r="J3" t="str">
         <v>Alexandria</v>
@@ -525,25 +525,113 @@
         <v/>
       </c>
       <c r="L3" t="str">
-        <v>2026-02-01</v>
+        <v>2026-01-12</v>
       </c>
       <c r="M3" t="str">
         <v>Active</v>
       </c>
       <c r="N3" t="str">
+        <v>Demo: leadership + communication</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>TR-2026-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Omar Khalil Ibrahim</v>
+      </c>
+      <c r="C4" t="str">
+        <v>+20 102 444 5566</v>
+      </c>
+      <c r="D4" t="str">
+        <v>omar.khalil@example.org</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Corporate</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Delta Engineering S.A.E.</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Project Coordinator</v>
+      </c>
+      <c r="H4" t="str">
         <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>Operations</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Giza</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v>2026-01-20</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Demo: communication skills cohort</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>TR-2026-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Layla Farouk</v>
+      </c>
+      <c r="C5" t="str">
+        <v>+20 103 555 6677</v>
+      </c>
+      <c r="D5" t="str">
+        <v>layla.farouk@example.org</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Student</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>The American University in Cairo</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Business Administration</v>
+      </c>
+      <c r="J5" t="str">
+        <v>New Cairo</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v>2026-02-03</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Active</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Demo: summer intake</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -576,43 +664,101 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CR-SAMPLE01</v>
+        <v>CR-LEAD-101</v>
       </c>
       <c r="B2" t="str">
-        <v>Sample Course Title</v>
+        <v>Leadership Essentials for Healthcare Teams</v>
       </c>
       <c r="C2" t="str">
-        <v>Soft Skills</v>
+        <v>Leadership</v>
       </c>
       <c r="D2" t="str">
-        <v>Mixed</v>
+        <v>Clinical &amp; administrative staff</v>
       </c>
       <c r="E2" t="str">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="F2" t="str">
-        <v>Online</v>
+        <v>Hybrid</v>
       </c>
       <c r="G2" t="str">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="H2" t="str">
-        <v>Demonstration course row</v>
+        <v>Team communication, prioritization, and leading small-group improvement projects. Includes two onsite workshops.</v>
       </c>
       <c r="I2" t="str">
         <v>Active</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>CR-COMM-201</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Professional Communication &amp; Presentation</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Soft Skills</v>
+      </c>
+      <c r="D3" t="str">
+        <v>All professional tracks</v>
+      </c>
+      <c r="E3" t="str">
+        <v>16</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Online</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2800</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Structured messaging, slide design, and delivering concise briefings to senior stakeholders.</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>CR-QUAL-301</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Quality Improvement in Clinical Settings</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Quality</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Physicians, nurses, quality officers</v>
+      </c>
+      <c r="E4" t="str">
+        <v>32</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Hybrid</v>
+      </c>
+      <c r="G4" t="str">
+        <v>6200</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Introduction to PDSA cycles, indicators, and audit-ready documentation for hospital units.</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Active</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -642,40 +788,92 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BA-SAMPLE01</v>
+        <v>BA-2026-Q1-LEAD</v>
       </c>
       <c r="B2" t="str">
-        <v>CR-SAMPLE01</v>
+        <v>CR-LEAD-101</v>
       </c>
       <c r="C2" t="str">
-        <v>Sample Batch 01</v>
+        <v>Leadership Cohort — Q1 2026 Cairo</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-03-01</v>
+        <v>2026-03-02</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-06-30</v>
+        <v>2026-05-15</v>
       </c>
       <c r="F2" t="str">
-        <v>Sample Trainer</v>
+        <v>Dr. Amira Soliman</v>
       </c>
       <c r="G2" t="str">
-        <v>Cairo</v>
+        <v>SBS Training Center — Cairo</v>
       </c>
       <c r="H2" t="str">
-        <v>25</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>BA-2026-Q1-COMM</v>
+      </c>
+      <c r="B3" t="str">
+        <v>CR-COMM-201</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Communication Skills — March Intake</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-03-10</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-04-20</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Ms. Dina Kamel</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Online (live sessions)</v>
+      </c>
+      <c r="H3" t="str">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>BA-2026-H1-QUAL</v>
+      </c>
+      <c r="B4" t="str">
+        <v>CR-QUAL-301</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Quality Improvement — H1 2026</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-04-07</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Dr. Hany Mourad</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Cairo + site visits</v>
+      </c>
+      <c r="H4" t="str">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -708,36 +906,152 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EN-SAMPLE01</v>
+        <v>EN-2026-0001</v>
       </c>
       <c r="B2" t="str">
-        <v>TR-SAMPLE01</v>
+        <v>TR-2026-001</v>
       </c>
       <c r="C2" t="str">
-        <v>BA-SAMPLE01</v>
+        <v>BA-2026-Q1-LEAD</v>
       </c>
       <c r="D2" t="str">
         <v>Registered</v>
       </c>
       <c r="E2" t="str">
-        <v>Pending</v>
+        <v>Paid</v>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>4500</v>
       </c>
       <c r="G2" t="str">
         <v>No</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-04-01</v>
+        <v>2026-02-10</v>
       </c>
       <c r="I2" t="str">
-        <v>Links sample trainee and batch</v>
+        <v>Physician track — full fee received</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EN-2026-0002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TR-2026-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>BA-2026-Q1-LEAD</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2250</v>
+      </c>
+      <c r="G3" t="str">
+        <v>No</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-02-11</v>
+      </c>
+      <c r="I3" t="str">
+        <v>50% deposit received; balance due before first workshop</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>EN-2026-0003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>TR-2026-003</v>
+      </c>
+      <c r="C4" t="str">
+        <v>BA-2026-Q1-COMM</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Attended</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2800</v>
+      </c>
+      <c r="G4" t="str">
+        <v>No</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-02-15</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Corporate-sponsored enrollment</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>EN-2026-0004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>TR-2026-004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>BA-2026-Q1-COMM</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>No</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2026-02-18</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Awaiting student discount approval</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>EN-2026-0005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>TR-2026-001</v>
+      </c>
+      <c r="C6" t="str">
+        <v>BA-2026-H1-QUAL</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Registered</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>No</v>
+      </c>
+      <c r="H6" t="str">
+        <v>2026-02-20</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Second program for same trainee; payment plan TBD</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>